<commit_message>
Added 2022-23 CO3I OOP paper found entry in sheet
</commit_message>
<xml_diff>
--- a/UT1 AND UT2 PAPER FOUND.xlsx
+++ b/UT1 AND UT2 PAPER FOUND.xlsx
@@ -1,22 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSBTE-28\Documents\ada\gpd_nba\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{472D0449-614A-4BFF-8578-E0B71078B9D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="Z_B61AD973_B989_4EFF_8A15_DB8242DBA907_.wvu.FilterData">Sheet1!$A$2:$F$12</definedName>
+    <definedName name="Z_B61AD973_B989_4EFF_8A15_DB8242DBA907_.wvu.FilterData" localSheetId="0" hidden="1">Sheet1!$A$2:$F$13</definedName>
   </definedNames>
-  <calcPr/>
+  <calcPr calcId="0"/>
   <customWorkbookViews>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{B61AD973-B989-4EFF-8A15-DB8242DBA907}" name="Group by AY"/>
+    <customWorkbookView name="Group by AY" guid="{B61AD973-B989-4EFF-8A15-DB8242DBA907}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
   </customWorkbookViews>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="26">
   <si>
     <t>Sr. No</t>
   </si>
@@ -91,21 +101,24 @@
   </si>
   <si>
     <t>2025-26</t>
+  </si>
+  <si>
+    <t>OOP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Verdana"/>
     </font>
@@ -115,7 +128,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -149,7 +162,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -163,75 +182,37 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="6" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF356854"/>
-          <bgColor rgb="FF356854"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <border>
         <left style="thin">
@@ -248,42 +229,69 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF356854"/>
+          <bgColor rgb="FF356854"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="Sheet1-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="Sheet1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A2:F12" displayName="Table1" name="Table1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A2:F13">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F13">
+    <sortCondition ref="B2:B13"/>
+  </sortState>
   <tableColumns count="6">
-    <tableColumn name="Sr. No" id="1"/>
-    <tableColumn name="AY" id="2"/>
-    <tableColumn name="SEM/SCHEME" id="3"/>
-    <tableColumn name="Program" id="4"/>
-    <tableColumn name="Test" id="5"/>
-    <tableColumn name="Test 2" id="6"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Sr. No"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="AY"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="SEM/SCHEME"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Program"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Test"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Test 2"/>
   </tableColumns>
-  <tableStyleInfo name="Sheet1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Sheet1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -473,26 +481,29 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A2:F13"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="13.38"/>
-    <col customWidth="1" min="2" max="2" width="27.75"/>
-    <col customWidth="1" min="3" max="3" width="24.88"/>
-    <col customWidth="1" min="4" max="4" width="23.0"/>
-    <col customWidth="1" min="5" max="5" width="18.75"/>
-    <col customWidth="1" min="6" max="6" width="15.25"/>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" customWidth="1"/>
+    <col min="4" max="4" width="23" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="30.75" customHeight="1">
+    <row r="2" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -512,9 +523,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
+    <row r="3" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>6</v>
@@ -532,9 +543,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
+    <row r="4" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>6</v>
@@ -552,78 +563,78 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
+    <row r="5" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
-        <v>4.0</v>
+        <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
+      <c r="E7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
-        <v>6.0</v>
+        <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>9</v>
@@ -632,18 +643,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
+    <row r="9" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
-        <v>7.0</v>
+        <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>9</v>
@@ -652,78 +663,98 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
+    <row r="10" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
-        <v>8.0</v>
+        <v>7</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="4">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" s="5" t="s">
+      <c r="E11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="6">
-        <v>9.0</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" ht="22.5" customHeight="1">
+    <row r="12" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
-        <v>10.0</v>
+        <v>9</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="6">
+        <v>10</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D13" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" s="6" t="s">
+      <c r="E13" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <customSheetViews>
     <customSheetView guid="{B61AD973-B989-4EFF-8A15-DB8242DBA907}" filter="1" showAutoFilter="1">
-      <autoFilter ref="$A$2:$F$12"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <autoFilter ref="A2:F12" xr:uid="{CEAC54D5-A9E8-40FC-BDF5-DC540CF0B32A}"/>
     </customSheetView>
   </customSheetViews>
-  <printOptions gridLines="1" horizontalCentered="1"/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup fitToHeight="0" cellComments="atEnd" orientation="landscape" pageOrder="overThenDown"/>
-  <drawing r:id="rId1"/>
+  <printOptions horizontalCentered="1" gridLines="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup fitToHeight="0" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>